<commit_message>
Refine Tower canvas and refresh template
</commit_message>
<xml_diff>
--- a/docs/build/tower-ai-program-template/AI_Program_Tracking_Template_Tower_v1.xlsx
+++ b/docs/build/tower-ai-program-template/AI_Program_Tracking_Template_Tower_v1.xlsx
@@ -2,18 +2,19 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rac47cf5ebd6543b9"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Register" sheetId="2" r:id="Rb311cfaae20c46ad"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category Playbooks" sheetId="3" r:id="Re7bea8930b614158"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tower Setup Upload" sheetId="4" r:id="Rcb38d4976a504f87"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Dictionary" sheetId="5" r:id="Rb2d08772ba6f40a7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI History" sheetId="6" r:id="R2580b422c3884961"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendors and Renewals" sheetId="7" r:id="Rddfa5bae32eb4f6f"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R10eb636357854ad0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stakeholder Notes" sheetId="9" r:id="R213452209f884f0c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="10" r:id="R63b27f2d3d9f409b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tower Mapping" sheetId="11" r:id="Rab3b1c8e4e9344b5"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="12" r:id="R3e1981249aa946bb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Rd7c702fb0738485a"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Register" sheetId="2" r:id="R4cf22063e6c84bd4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category Playbooks" sheetId="3" r:id="R4aad88b6f46f4cd7"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tower Setup Upload" sheetId="4" r:id="R105a91db31064113"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Dictionary" sheetId="5" r:id="Rd5acf11ed1164634"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI History" sheetId="6" r:id="Re930d347d4f348ba"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendors and Renewals" sheetId="7" r:id="Rda18195624564e54"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="8" r:id="R31e05a99460f4f70"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stakeholder Notes" sheetId="9" r:id="R3951bac493334304"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="10" r:id="R26f9e1eca5a94586"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard Feed Map" sheetId="11" r:id="R4b59482110384e16"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tower Mapping" sheetId="12" r:id="R221960c4f80749cc"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="13" r:id="R6dd0aa6db49a4c57"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -258,17 +259,25 @@
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Tower DB mapping</x:v>
+        <x:v>Refresh posture</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>ai_initiatives, ai_initiative_kpis, ai_initiative_vendors, ai_initiative_decisions, ai_initiative_stakeholder_notes, ai_initiative_scenarios.</x:v>
+        <x:v>Pilot operating rhythm is weekly refresh. Future operating rhythm is daily refresh through APIs, S3 drops, or scheduled file exports. Dashboards update from parsed DB rows, not directly from workbook cells.</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
+        <x:v>Tower DB mapping</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>ai_initiatives, ai_initiative_kpis, ai_initiative_vendors, ai_initiative_decisions, ai_initiative_stakeholder_notes, ai_initiative_scenarios.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
         <x:v>Confidence rule</x:v>
       </x:c>
-      <x:c r="B6" t="str">
+      <x:c r="B7" t="str">
         <x:v>HIGH = system extract or signed governance artifact. MED = owner-attested spreadsheet or current workshop note. LOW = draft estimate or incomplete source.</x:v>
       </x:c>
     </x:row>
@@ -422,162 +431,321 @@
   <x:sheetData>
     <x:row r="1">
       <x:c r="A1" t="str">
-        <x:v>Tower page/lens</x:v>
+        <x:v>dashboard_area</x:v>
       </x:c>
       <x:c r="B1" t="str">
-        <x:v>Question it should answer</x:v>
+        <x:v>dashboard_metric_or_view</x:v>
       </x:c>
       <x:c r="C1" t="str">
-        <x:v>Minimum data needed</x:v>
+        <x:v>source_sheet</x:v>
       </x:c>
       <x:c r="D1" t="str">
-        <x:v>Best data needed</x:v>
+        <x:v>db_target</x:v>
       </x:c>
       <x:c r="E1" t="str">
-        <x:v>Manual allowed?</x:v>
+        <x:v>current_refresh_cycle</x:v>
       </x:c>
       <x:c r="F1" t="str">
-        <x:v>What not to claim</x:v>
+        <x:v>future_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="G1" t="str">
+        <x:v>update_trigger</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>source_system_examples</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>cxo_provenance_question</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
       <x:c r="A2" t="str">
-        <x:v>Portfolio</x:v>
+        <x:v>KPI band</x:v>
       </x:c>
       <x:c r="B2" t="str">
-        <x:v>Where is the portfolio positioned against value and strategy?</x:v>
+        <x:v>Portfolio ROI</x:v>
       </x:c>
       <x:c r="C2" t="str">
-        <x:v>Initiative registry with stage, status, committed, measured.</x:v>
+        <x:v>Program Register + KPI History</x:v>
       </x:c>
       <x:c r="D2" t="str">
-        <x:v>KPI history, alignment rationale, confidence, strategic goal mapping.</x:v>
+        <x:v>ai_initiatives + ai_initiative_kpis</x:v>
       </x:c>
       <x:c r="E2" t="str">
-        <x:v>Yes for strategy mapping</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="F2" t="str">
-        <x:v>Do not imply ROI for foundation programs without measured value.</x:v>
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="G2" t="str">
+        <x:v>Refresh after committed value and measured value are validated and committed.</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>Finance benefits tracker, BI semantic layer, business case workbook</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>Which finance source produced measured value, and who signed confidence?</x:v>
       </x:c>
     </x:row>
     <x:row r="3">
       <x:c r="A3" t="str">
-        <x:v>Scorecards / Value</x:v>
+        <x:v>KPI band</x:v>
       </x:c>
       <x:c r="B3" t="str">
-        <x:v>Which initiatives are furthest from earning their commitment?</x:v>
+        <x:v>Active pressures</x:v>
       </x:c>
       <x:c r="C3" t="str">
-        <x:v>Committed and measured value.</x:v>
+        <x:v>Program Register + Decisions + KPI History</x:v>
       </x:c>
       <x:c r="D3" t="str">
-        <x:v>Quarterly KPI history with finance signoff and peer median.</x:v>
+        <x:v>ai_initiatives + ai_initiative_decisions + ai_initiative_kpis</x:v>
       </x:c>
       <x:c r="E3" t="str">
-        <x:v>Limited</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="F3" t="str">
-        <x:v>Do not treat activity as value.</x:v>
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="G3" t="str">
+        <x:v>Refresh after status_flag, owner, and current evidence are committed.</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>PMO portfolio export, steering log, KPI workbook</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>What changed this week that made this a pressure?</x:v>
       </x:c>
     </x:row>
     <x:row r="4">
       <x:c r="A4" t="str">
-        <x:v>Scorecards / Adoption</x:v>
+        <x:v>KPI band</x:v>
       </x:c>
       <x:c r="B4" t="str">
-        <x:v>Where is adoption blocking value conversion?</x:v>
+        <x:v>Spend at risk</x:v>
       </x:c>
       <x:c r="C4" t="str">
-        <x:v>Status flag and stage.</x:v>
+        <x:v>Program Register + Vendors and Renewals</x:v>
       </x:c>
       <x:c r="D4" t="str">
-        <x:v>Usage cohort, eligible population, training, workflow fit, stakeholder blockers.</x:v>
+        <x:v>ai_initiatives + ai_initiative_vendors</x:v>
       </x:c>
       <x:c r="E4" t="str">
-        <x:v>Yes for blockers</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="F4" t="str">
-        <x:v>Do not label vendor as blocker without user/workflow evidence.</x:v>
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="G4" t="str">
+        <x:v>Refresh after committed spend and vendor rows are validated.</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Budget system, vendor master, contract register</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>Which spend is exposed, and is it spend, value, or contract risk?</x:v>
       </x:c>
     </x:row>
     <x:row r="5">
       <x:c r="A5" t="str">
-        <x:v>Gates</x:v>
+        <x:v>KPI band</x:v>
       </x:c>
       <x:c r="B5" t="str">
-        <x:v>Which lifecycle stage needs a decision?</x:v>
+        <x:v>Renewals in 90 days</x:v>
       </x:c>
       <x:c r="C5" t="str">
-        <x:v>Stage, decision status, owner.</x:v>
+        <x:v>Vendors and Renewals</x:v>
       </x:c>
       <x:c r="D5" t="str">
-        <x:v>Decision history, dissent, next gate criteria, outcome status.</x:v>
+        <x:v>ai_initiative_vendors</x:v>
       </x:c>
       <x:c r="E5" t="str">
-        <x:v>Yes</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="F5" t="str">
-        <x:v>Do not invent missing phases.</x:v>
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="G5" t="str">
+        <x:v>Refresh after renewal calendar import and contract owner validation.</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Coupa, Ariba, Ironclad, procurement calendar</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>What contract register fed the date and value?</x:v>
       </x:c>
     </x:row>
     <x:row r="6">
       <x:c r="A6" t="str">
-        <x:v>Dependencies / Contract</x:v>
+        <x:v>KPI band</x:v>
       </x:c>
       <x:c r="B6" t="str">
-        <x:v>Which vendor decisions are time-sensitive?</x:v>
+        <x:v>Adoption</x:v>
       </x:c>
       <x:c r="C6" t="str">
-        <x:v>Vendor, contract value, renewal date.</x:v>
+        <x:v>KPI History + Stakeholder Notes</x:v>
       </x:c>
       <x:c r="D6" t="str">
-        <x:v>Usage evidence, renewal thesis, vendor health, procurement owner.</x:v>
+        <x:v>ai_initiative_kpis + ai_initiative_stakeholder_notes</x:v>
       </x:c>
       <x:c r="E6" t="str">
-        <x:v>Some</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="F6" t="str">
-        <x:v>Do not equate renewal date with value.</x:v>
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="G6" t="str">
+        <x:v>Refresh after usage, eligible population, training, and blocker notes are joined.</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>M365 admin, GitHub, ServiceNow, LMS, survey notes</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Is adoption based on real usage, training completion, or owner attestation?</x:v>
       </x:c>
     </x:row>
     <x:row r="7">
       <x:c r="A7" t="str">
-        <x:v>Dependencies / Risk</x:v>
+        <x:v>Portfolio canvas</x:v>
       </x:c>
       <x:c r="B7" t="str">
-        <x:v>Which third-party relationship amplifies portfolio risk?</x:v>
+        <x:v>Today's pressures</x:v>
       </x:c>
       <x:c r="C7" t="str">
-        <x:v>Vendor health and owning initiative status.</x:v>
+        <x:v>Program Register + KPI History + Vendors and Renewals + Decisions</x:v>
       </x:c>
       <x:c r="D7" t="str">
-        <x:v>Security review, incident history, financial health, dependency criticality.</x:v>
+        <x:v>ai_initiatives + ai_initiative_kpis + ai_initiative_vendors + ai_initiative_decisions</x:v>
       </x:c>
       <x:c r="E7" t="str">
-        <x:v>Some</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="F7" t="str">
-        <x:v>Do not call moderate health high risk without supporting evidence.</x:v>
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="G7" t="str">
+        <x:v>Refresh after parser commits all validated rows for the tenant.</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>PMO, Finance, Procurement, BI, governance log</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>Which rows produced this pressure and what is missing?</x:v>
       </x:c>
     </x:row>
     <x:row r="8">
       <x:c r="A8" t="str">
+        <x:v>Portfolio canvas</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>Strategic alignment 2x2</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Program Register + KPI History</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>ai_initiatives + ai_initiative_kpis</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="G8" t="str">
+        <x:v>Refresh after measured value, confidence, and strategy alignment fields are committed.</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>Strategy plan, benefits tracker, PMO intake</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>Is matrix placement value-backed or strategy-attested?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9">
+      <x:c r="A9" t="str">
+        <x:v>Portfolio canvas</x:v>
+      </x:c>
+      <x:c r="B9" t="str">
+        <x:v>Evidence map</x:v>
+      </x:c>
+      <x:c r="C9" t="str">
+        <x:v>All sheets + supporting files</x:v>
+      </x:c>
+      <x:c r="D9" t="str">
+        <x:v>uploaded_files + data_uploads + AI registry tables + corpus chunks</x:v>
+      </x:c>
+      <x:c r="E9" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="F9" t="str">
+        <x:v>Daily API/export or S3 drop</x:v>
+      </x:c>
+      <x:c r="G9" t="str">
+        <x:v>Refresh after upload is classified, parsed, chunked, and linked to initiatives.</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>Tower setup upload, S3 bucket, vendor exports</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
+        <x:v>Which uploads were parsed, which need mapping, and what dashboards changed?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10">
+      <x:c r="A10" t="str">
+        <x:v>Dependencies</x:v>
+      </x:c>
+      <x:c r="B10" t="str">
+        <x:v>Vendor dependency ranking</x:v>
+      </x:c>
+      <x:c r="C10" t="str">
+        <x:v>Vendors and Renewals + Program Register + KPI History</x:v>
+      </x:c>
+      <x:c r="D10" t="str">
+        <x:v>ai_initiative_vendors + ai_initiatives + ai_initiative_kpis</x:v>
+      </x:c>
+      <x:c r="E10" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="F10" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="G10" t="str">
+        <x:v>Refresh after vendor health, renewal date, initiative status, and adoption/value evidence are joined.</x:v>
+      </x:c>
+      <x:c r="H10" t="str">
+        <x:v>Procurement system, vendor admin console, PMO register, usage export</x:v>
+      </x:c>
+      <x:c r="I10" t="str">
+        <x:v>Is this dependency ranked by contract timing, value risk, adoption blocker, or vendor health?</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11">
+      <x:c r="A11" t="str">
         <x:v>Executive brief</x:v>
       </x:c>
-      <x:c r="B8" t="str">
-        <x:v>What should the board or CXO decide next?</x:v>
-      </x:c>
-      <x:c r="C8" t="str">
-        <x:v>Initiatives, pressure cards, vendors, confidence.</x:v>
-      </x:c>
-      <x:c r="D8" t="str">
-        <x:v>All evidence feeds with source artifact and owner.</x:v>
-      </x:c>
-      <x:c r="E8" t="str">
-        <x:v>Yes for narrative</x:v>
-      </x:c>
-      <x:c r="F8" t="str">
-        <x:v>Do not cite private quotes without attribution consent.</x:v>
+      <x:c r="B11" t="str">
+        <x:v>Board read and one thing today</x:v>
+      </x:c>
+      <x:c r="C11" t="str">
+        <x:v>All validated sheets</x:v>
+      </x:c>
+      <x:c r="D11" t="str">
+        <x:v>AI registry tables + corpus chunks + graph links</x:v>
+      </x:c>
+      <x:c r="E11" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="F11" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="G11" t="str">
+        <x:v>Refresh after all feeds pass import checks and Atlas synthesis uses row-level citations.</x:v>
+      </x:c>
+      <x:c r="H11" t="str">
+        <x:v>Validated Tower setup import</x:v>
+      </x:c>
+      <x:c r="I11" t="str">
+        <x:v>What evidence supports the recommendation, and what is deferred?</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
@@ -586,6 +754,175 @@
 </file>
 
 <file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:sheetData>
+    <x:row r="1">
+      <x:c r="A1" t="str">
+        <x:v>Tower page/lens</x:v>
+      </x:c>
+      <x:c r="B1" t="str">
+        <x:v>Question it should answer</x:v>
+      </x:c>
+      <x:c r="C1" t="str">
+        <x:v>Minimum data needed</x:v>
+      </x:c>
+      <x:c r="D1" t="str">
+        <x:v>Best data needed</x:v>
+      </x:c>
+      <x:c r="E1" t="str">
+        <x:v>Manual allowed?</x:v>
+      </x:c>
+      <x:c r="F1" t="str">
+        <x:v>What not to claim</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str">
+        <x:v>Portfolio</x:v>
+      </x:c>
+      <x:c r="B2" t="str">
+        <x:v>Where is the portfolio positioned against value and strategy?</x:v>
+      </x:c>
+      <x:c r="C2" t="str">
+        <x:v>Initiative registry with stage, status, committed, measured.</x:v>
+      </x:c>
+      <x:c r="D2" t="str">
+        <x:v>KPI history, alignment rationale, confidence, strategic goal mapping.</x:v>
+      </x:c>
+      <x:c r="E2" t="str">
+        <x:v>Yes for strategy mapping</x:v>
+      </x:c>
+      <x:c r="F2" t="str">
+        <x:v>Do not imply ROI for foundation programs without measured value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="3">
+      <x:c r="A3" t="str">
+        <x:v>Scorecards / Value</x:v>
+      </x:c>
+      <x:c r="B3" t="str">
+        <x:v>Which initiatives are furthest from earning their commitment?</x:v>
+      </x:c>
+      <x:c r="C3" t="str">
+        <x:v>Committed and measured value.</x:v>
+      </x:c>
+      <x:c r="D3" t="str">
+        <x:v>Quarterly KPI history with finance signoff and peer median.</x:v>
+      </x:c>
+      <x:c r="E3" t="str">
+        <x:v>Limited</x:v>
+      </x:c>
+      <x:c r="F3" t="str">
+        <x:v>Do not treat activity as value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4">
+      <x:c r="A4" t="str">
+        <x:v>Scorecards / Adoption</x:v>
+      </x:c>
+      <x:c r="B4" t="str">
+        <x:v>Where is adoption blocking value conversion?</x:v>
+      </x:c>
+      <x:c r="C4" t="str">
+        <x:v>Status flag and stage.</x:v>
+      </x:c>
+      <x:c r="D4" t="str">
+        <x:v>Usage cohort, eligible population, training, workflow fit, stakeholder blockers.</x:v>
+      </x:c>
+      <x:c r="E4" t="str">
+        <x:v>Yes for blockers</x:v>
+      </x:c>
+      <x:c r="F4" t="str">
+        <x:v>Do not label vendor as blocker without user/workflow evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" t="str">
+        <x:v>Gates</x:v>
+      </x:c>
+      <x:c r="B5" t="str">
+        <x:v>Which lifecycle stage needs a decision?</x:v>
+      </x:c>
+      <x:c r="C5" t="str">
+        <x:v>Stage, decision status, owner.</x:v>
+      </x:c>
+      <x:c r="D5" t="str">
+        <x:v>Decision history, dissent, next gate criteria, outcome status.</x:v>
+      </x:c>
+      <x:c r="E5" t="str">
+        <x:v>Yes</x:v>
+      </x:c>
+      <x:c r="F5" t="str">
+        <x:v>Do not invent missing phases.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" t="str">
+        <x:v>Dependencies / Contract</x:v>
+      </x:c>
+      <x:c r="B6" t="str">
+        <x:v>Which vendor decisions are time-sensitive?</x:v>
+      </x:c>
+      <x:c r="C6" t="str">
+        <x:v>Vendor, contract value, renewal date.</x:v>
+      </x:c>
+      <x:c r="D6" t="str">
+        <x:v>Usage evidence, renewal thesis, vendor health, procurement owner.</x:v>
+      </x:c>
+      <x:c r="E6" t="str">
+        <x:v>Some</x:v>
+      </x:c>
+      <x:c r="F6" t="str">
+        <x:v>Do not equate renewal date with value.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" t="str">
+        <x:v>Dependencies / Risk</x:v>
+      </x:c>
+      <x:c r="B7" t="str">
+        <x:v>Which third-party relationship amplifies portfolio risk?</x:v>
+      </x:c>
+      <x:c r="C7" t="str">
+        <x:v>Vendor health and owning initiative status.</x:v>
+      </x:c>
+      <x:c r="D7" t="str">
+        <x:v>Security review, incident history, financial health, dependency criticality.</x:v>
+      </x:c>
+      <x:c r="E7" t="str">
+        <x:v>Some</x:v>
+      </x:c>
+      <x:c r="F7" t="str">
+        <x:v>Do not call moderate health high risk without supporting evidence.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" t="str">
+        <x:v>Executive brief</x:v>
+      </x:c>
+      <x:c r="B8" t="str">
+        <x:v>What should the board or CXO decide next?</x:v>
+      </x:c>
+      <x:c r="C8" t="str">
+        <x:v>Initiatives, pressure cards, vendors, confidence.</x:v>
+      </x:c>
+      <x:c r="D8" t="str">
+        <x:v>All evidence feeds with source artifact and owner.</x:v>
+      </x:c>
+      <x:c r="E8" t="str">
+        <x:v>Yes for narrative</x:v>
+      </x:c>
+      <x:c r="F8" t="str">
+        <x:v>Do not cite private quotes without attribution consent.</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:sheetData>
@@ -756,15 +1093,21 @@
         <x:v>manual_allowed</x:v>
       </x:c>
       <x:c r="S1" t="str">
-        <x:v>refresh_cadence</x:v>
+        <x:v>current_refresh_cycle</x:v>
       </x:c>
       <x:c r="T1" t="str">
+        <x:v>future_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="U1" t="str">
+        <x:v>dashboard_update_rule</x:v>
+      </x:c>
+      <x:c r="V1" t="str">
         <x:v>tower_pages_supported</x:v>
       </x:c>
-      <x:c r="U1" t="str">
+      <x:c r="W1" t="str">
         <x:v>next_missing_evidence</x:v>
       </x:c>
-      <x:c r="V1" t="str">
+      <x:c r="X1" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
@@ -824,15 +1167,21 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S2" t="str">
-        <x:v>Weekly during pilot</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="T2" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="U2" t="str">
+        <x:v>Refresh KPI/adoption dashboard after ai_initiative_kpis and status_flag are committed.</x:v>
+      </x:c>
+      <x:c r="V2" t="str">
         <x:v>Portfolio; Scorecards; Gates; Dependencies; Executive brief</x:v>
       </x:c>
-      <x:c r="U2" t="str">
+      <x:c r="W2" t="str">
         <x:v>Active users by cohort and training completion by store</x:v>
       </x:c>
-      <x:c r="V2" t="str">
+      <x:c r="X2" t="str">
         <x:v>Example row</x:v>
       </x:c>
     </x:row>
@@ -892,15 +1241,21 @@
         <x:v>Some</x:v>
       </x:c>
       <x:c r="S3" t="str">
-        <x:v>Monthly</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="T3" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="U3" t="str">
+        <x:v>Refresh value/adoption tiles after delivery metrics and quality guardrails are committed.</x:v>
+      </x:c>
+      <x:c r="V3" t="str">
         <x:v>Scorecards; Dependencies; Executive brief</x:v>
       </x:c>
-      <x:c r="U3" t="str">
+      <x:c r="W3" t="str">
         <x:v>Quality and security review trend</x:v>
       </x:c>
-      <x:c r="V3" t="str">
+      <x:c r="X3" t="str">
         <x:v>Example row</x:v>
       </x:c>
     </x:row>
@@ -963,12 +1318,18 @@
         <x:v>Weekly</x:v>
       </x:c>
       <x:c r="T4" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="U4" t="str">
+        <x:v>Refresh scorecards when containment, escalation, CSAT, and cost metrics are committed.</x:v>
+      </x:c>
+      <x:c r="V4" t="str">
         <x:v>Portfolio; Scorecards; Dependencies; Executive brief</x:v>
       </x:c>
-      <x:c r="U4" t="str">
+      <x:c r="W4" t="str">
         <x:v>Containment, escalation, CSAT, risk review</x:v>
       </x:c>
-      <x:c r="V4" t="str">
+      <x:c r="X4" t="str">
         <x:v>Example row</x:v>
       </x:c>
     </x:row>
@@ -1028,15 +1389,21 @@
         <x:v>Some</x:v>
       </x:c>
       <x:c r="S5" t="str">
-        <x:v>Monthly</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="T5" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="U5" t="str">
+        <x:v>Refresh dependency/contract views after usage, process KPI, and renewal evidence are committed.</x:v>
+      </x:c>
+      <x:c r="V5" t="str">
         <x:v>Dependencies; Contract lens; Executive brief</x:v>
       </x:c>
-      <x:c r="U5" t="str">
+      <x:c r="W5" t="str">
         <x:v>Renewal thesis and adoption baseline</x:v>
       </x:c>
-      <x:c r="V5" t="str">
+      <x:c r="X5" t="str">
         <x:v>Example row</x:v>
       </x:c>
     </x:row>
@@ -1096,15 +1463,21 @@
         <x:v>Some</x:v>
       </x:c>
       <x:c r="S6" t="str">
-        <x:v>Weekly during pilot</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="T6" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="U6" t="str">
+        <x:v>Refresh adoption and operational pressure cards after ITSM deflection/reopen/SLA rows are committed.</x:v>
+      </x:c>
+      <x:c r="V6" t="str">
         <x:v>Scorecards; Dependencies; Executive brief</x:v>
       </x:c>
-      <x:c r="U6" t="str">
+      <x:c r="W6" t="str">
         <x:v>Deflection by category and escalation quality</x:v>
       </x:c>
-      <x:c r="V6" t="str">
+      <x:c r="X6" t="str">
         <x:v>Example row</x:v>
       </x:c>
     </x:row>
@@ -1164,15 +1537,21 @@
         <x:v>Yes</x:v>
       </x:c>
       <x:c r="S7" t="str">
-        <x:v>Monthly</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="T7" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="U7" t="str">
+        <x:v>Refresh foundation/evidence view after coverage, SLO, and cost-tagging metrics are committed.</x:v>
+      </x:c>
+      <x:c r="V7" t="str">
         <x:v>Gates; Scorecards; Executive brief</x:v>
       </x:c>
-      <x:c r="U7" t="str">
+      <x:c r="W7" t="str">
         <x:v>Cost allocation coverage and tagged model usage</x:v>
       </x:c>
-      <x:c r="V7" t="str">
+      <x:c r="X7" t="str">
         <x:v>Example row</x:v>
       </x:c>
     </x:row>
@@ -1232,15 +1611,21 @@
         <x:v>Some</x:v>
       </x:c>
       <x:c r="S8" t="str">
-        <x:v>Monthly</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="T8" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="U8" t="str">
+        <x:v>Refresh value/adoption dashboard after cycle-time, release quality, and outcome rows are committed.</x:v>
+      </x:c>
+      <x:c r="V8" t="str">
         <x:v>Portfolio; Scorecards; Executive brief</x:v>
       </x:c>
-      <x:c r="U8" t="str">
+      <x:c r="W8" t="str">
         <x:v>Outcome quality, cycle time, and release safety evidence</x:v>
       </x:c>
-      <x:c r="V8" t="str">
+      <x:c r="X8" t="str">
         <x:v>Example row</x:v>
       </x:c>
     </x:row>
@@ -1273,9 +1658,15 @@
         <x:v>manual_inputs_allowed</x:v>
       </x:c>
       <x:c r="G1" t="str">
+        <x:v>current_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>future_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
         <x:v>collection_guidance_for_IT</x:v>
       </x:c>
-      <x:c r="H1" t="str">
+      <x:c r="J1" t="str">
         <x:v>Tower_interpretation</x:v>
       </x:c>
     </x:row>
@@ -1299,9 +1690,15 @@
         <x:v>Yes: workflow mapping, value hypothesis, blocker themes.</x:v>
       </x:c>
       <x:c r="G2" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
         <x:v>Export usage by user/cohort weekly. Join to eligible population and training roster. Capture blockers from store/team leads.</x:v>
       </x:c>
-      <x:c r="H2" t="str">
+      <x:c r="J2" t="str">
         <x:v>Adoption Gap means usage/training/workflow evidence is below target, not that the vendor is bad.</x:v>
       </x:c>
     </x:row>
@@ -1325,9 +1722,15 @@
         <x:v>Yes: team taxonomy and perceived productivity.</x:v>
       </x:c>
       <x:c r="G3" t="str">
-        <x:v>Pull GitHub Copilot metrics and engineering delivery metrics monthly. Do not claim value without baseline and quality check.</x:v>
+        <x:v>Weekly</x:v>
       </x:c>
       <x:c r="H3" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>Pull GitHub Copilot metrics and engineering delivery metrics weekly in pilot. Do not claim value without baseline and quality check.</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
         <x:v>Healthy requires both usage and quality/guardrail evidence.</x:v>
       </x:c>
     </x:row>
@@ -1351,9 +1754,15 @@
         <x:v>Some: risk notes, governance decisions.</x:v>
       </x:c>
       <x:c r="G4" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
         <x:v>Start with process volume and outcome baseline. Add model/control logs only after workflow is live.</x:v>
       </x:c>
-      <x:c r="H4" t="str">
+      <x:c r="J4" t="str">
         <x:v>Value Lag means the workflow is operating but has not converted into measured business outcome.</x:v>
       </x:c>
     </x:row>
@@ -1377,9 +1786,15 @@
         <x:v>Yes: process map, control judgement, value hypothesis.</x:v>
       </x:c>
       <x:c r="G5" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
         <x:v>Start with one process family. Export pre/post process KPIs and enabled agent capability. Join to controls and renewal exposure.</x:v>
       </x:c>
-      <x:c r="H5" t="str">
+      <x:c r="J5" t="str">
         <x:v>Tower should separate workflow adoption and control readiness from vendor renewal timing.</x:v>
       </x:c>
     </x:row>
@@ -1403,9 +1818,15 @@
         <x:v>Some: taxonomy cleanup and knowledge quality review.</x:v>
       </x:c>
       <x:c r="G6" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
         <x:v>Export request categories, eligible volumes, agent-handled cases, escalations, SLA and reopen data weekly during pilot.</x:v>
       </x:c>
-      <x:c r="H6" t="str">
+      <x:c r="J6" t="str">
         <x:v>Adoption Gap should mean the agent is not reliably used or trusted in the target service flow.</x:v>
       </x:c>
     </x:row>
@@ -1429,9 +1850,15 @@
         <x:v>Yes: workflow taxonomy and product outcome attribution.</x:v>
       </x:c>
       <x:c r="G7" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
         <x:v>Track by product/team, not just tool seats. Join AI usage to delivery flow and release quality. Require guardrail evidence before calling it scaled.</x:v>
       </x:c>
-      <x:c r="H7" t="str">
+      <x:c r="J7" t="str">
         <x:v>Healthy requires productivity plus release safety; value lag means usage exists but product/business outcome has not followed.</x:v>
       </x:c>
     </x:row>
@@ -1455,9 +1882,15 @@
         <x:v>Yes: target use case inventory and readiness scoring.</x:v>
       </x:c>
       <x:c r="G8" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
         <x:v>Treat as foundation until use cases consume it. Capture coverage and readiness, not ROI claims.</x:v>
       </x:c>
-      <x:c r="H8" t="str">
+      <x:c r="J8" t="str">
         <x:v>Foundation Phase should be separated from ROI programs in Tower 2x2.</x:v>
       </x:c>
     </x:row>
@@ -1481,9 +1914,15 @@
         <x:v>Yes: renewal thesis and business owner judgement.</x:v>
       </x:c>
       <x:c r="G9" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H9" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I9" t="str">
         <x:v>Join procurement renewal calendar to initiative owner and usage evidence. Do not treat renewal as value evidence.</x:v>
       </x:c>
-      <x:c r="H9" t="str">
+      <x:c r="J9" t="str">
         <x:v>Contract lens ranks timing and dollars; adoption/risk lens needs usage and control evidence.</x:v>
       </x:c>
     </x:row>
@@ -1516,9 +1955,18 @@
         <x:v>target_storage</x:v>
       </x:c>
       <x:c r="G1" t="str">
+        <x:v>current_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="H1" t="str">
+        <x:v>future_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="I1" t="str">
+        <x:v>dashboard_update_rule</x:v>
+      </x:c>
+      <x:c r="J1" t="str">
         <x:v>future_automation_path</x:v>
       </x:c>
-      <x:c r="H1" t="str">
+      <x:c r="K1" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
@@ -1542,9 +1990,18 @@
         <x:v>ai_initiatives</x:v>
       </x:c>
       <x:c r="G2" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H2" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I2" t="str">
+        <x:v>Refresh portfolio, gates, scorecards, and executive pressure cards after validated register rows are committed.</x:v>
+      </x:c>
+      <x:c r="J2" t="str">
         <x:v>API from PMO/PPM system</x:v>
       </x:c>
-      <x:c r="H2" t="str">
+      <x:c r="K2" t="str">
         <x:v>This is the anchor table. No Tower page should render a program without this row.</x:v>
       </x:c>
     </x:row>
@@ -1568,9 +2025,18 @@
         <x:v>ai_initiative_kpis + corpus chunks</x:v>
       </x:c>
       <x:c r="G3" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H3" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I3" t="str">
+        <x:v>Refresh value, adoption, and risk tiles after metric rows pass confidence checks.</x:v>
+      </x:c>
+      <x:c r="J3" t="str">
         <x:v>BI API or S3 drop with schema parser</x:v>
       </x:c>
-      <x:c r="H3" t="str">
+      <x:c r="K3" t="str">
         <x:v>KPI names can vary by category but must map to a standard metric family.</x:v>
       </x:c>
     </x:row>
@@ -1594,9 +2060,18 @@
         <x:v>ai_initiative_vendors + graph vendor nodes</x:v>
       </x:c>
       <x:c r="G4" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H4" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I4" t="str">
+        <x:v>Refresh dependencies, contract lens, 90-day renewal count, and spend-at-risk cards after renewal rows are committed.</x:v>
+      </x:c>
+      <x:c r="J4" t="str">
         <x:v>Coupa/Ariba/contract repository API</x:v>
       </x:c>
-      <x:c r="H4" t="str">
+      <x:c r="K4" t="str">
         <x:v>Renewal date alone is not value evidence.</x:v>
       </x:c>
     </x:row>
@@ -1620,9 +2095,18 @@
         <x:v>ai_initiative_decisions + graph decision nodes</x:v>
       </x:c>
       <x:c r="G5" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H5" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I5" t="str">
+        <x:v>Refresh gates and executive brief decision load after steering decisions are logged.</x:v>
+      </x:c>
+      <x:c r="J5" t="str">
         <x:v>Minutes parser or governance API</x:v>
       </x:c>
-      <x:c r="H5" t="str">
+      <x:c r="K5" t="str">
         <x:v>Dissent is useful evidence; it should not be erased.</x:v>
       </x:c>
     </x:row>
@@ -1646,9 +2130,18 @@
         <x:v>ai_initiative_stakeholder_notes + corpus chunks</x:v>
       </x:c>
       <x:c r="G6" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H6" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I6" t="str">
+        <x:v>Refresh adoption blockers, Atlas citations, and confidence context after notes are consent-checked.</x:v>
+      </x:c>
+      <x:c r="J6" t="str">
         <x:v>Survey/interview ingestion</x:v>
       </x:c>
-      <x:c r="H6" t="str">
+      <x:c r="K6" t="str">
         <x:v>Attribution consent is required before showing names or quotes.</x:v>
       </x:c>
     </x:row>
@@ -1672,9 +2165,18 @@
         <x:v>ai_initiative_scenarios + graph scenario nodes</x:v>
       </x:c>
       <x:c r="G7" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H7" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="I7" t="str">
+        <x:v>Refresh what-if answers and risk alternatives after probability and owner review.</x:v>
+      </x:c>
+      <x:c r="J7" t="str">
         <x:v>Risk register API or scenario workbook upload</x:v>
       </x:c>
-      <x:c r="H7" t="str">
+      <x:c r="K7" t="str">
         <x:v>Can start manual, then standardize later.</x:v>
       </x:c>
     </x:row>
@@ -1698,9 +2200,18 @@
         <x:v>object storage + corpus chunks + graph links</x:v>
       </x:c>
       <x:c r="G8" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="H8" t="str">
+        <x:v>Daily API/export or S3 drop</x:v>
+      </x:c>
+      <x:c r="I8" t="str">
+        <x:v>Refresh evidence map after files are classified, chunked, and linked to initiative rows.</x:v>
+      </x:c>
+      <x:c r="J8" t="str">
         <x:v>S3 bucket drop, event parser, vendor APIs</x:v>
       </x:c>
-      <x:c r="H8" t="str">
+      <x:c r="K8" t="str">
         <x:v>Every chunk should attach to tenant, initiative, source artifact, and confidence.</x:v>
       </x:c>
     </x:row>
@@ -2090,6 +2601,93 @@
         <x:v>What-if responses.</x:v>
       </x:c>
     </x:row>
+    <x:row r="14">
+      <x:c r="A14" t="str">
+        <x:v>current_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="B14" t="str">
+        <x:v>all intake sheets</x:v>
+      </x:c>
+      <x:c r="C14" t="str">
+        <x:v>source_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="D14" t="str">
+        <x:v>How often the tenant will refresh this feed during pilot operations.</x:v>
+      </x:c>
+      <x:c r="E14" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="F14" t="str">
+        <x:v>Template default with owner review</x:v>
+      </x:c>
+      <x:c r="G14" t="str">
+        <x:v>Weekly file upload, weekly extract</x:v>
+      </x:c>
+      <x:c r="H14" t="str">
+        <x:v>Default Weekly unless an owner provides a stricter cadence</x:v>
+      </x:c>
+      <x:c r="I14" t="str">
+        <x:v>Sets dashboard freshness label and import SLA.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="15">
+      <x:c r="A15" t="str">
+        <x:v>future_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="B15" t="str">
+        <x:v>all intake sheets</x:v>
+      </x:c>
+      <x:c r="C15" t="str">
+        <x:v>target_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="D15" t="str">
+        <x:v>Target cadence once API, S3, or scheduled exports replace manual uploads.</x:v>
+      </x:c>
+      <x:c r="E15" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="F15" t="str">
+        <x:v>Template default with architecture review</x:v>
+      </x:c>
+      <x:c r="G15" t="str">
+        <x:v>Vendor API, BI scheduled export, S3 drop</x:v>
+      </x:c>
+      <x:c r="H15" t="str">
+        <x:v>Default Daily API/export for operational feeds</x:v>
+      </x:c>
+      <x:c r="I15" t="str">
+        <x:v>Guides integration roadmap and stale-data warnings.</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="16">
+      <x:c r="A16" t="str">
+        <x:v>dashboard_update_rule</x:v>
+      </x:c>
+      <x:c r="B16" t="str">
+        <x:v>all intake sheets</x:v>
+      </x:c>
+      <x:c r="C16" t="str">
+        <x:v>dashboard_update_rule</x:v>
+      </x:c>
+      <x:c r="D16" t="str">
+        <x:v>Plain-English rule for when Tower can refresh the related dashboard elements.</x:v>
+      </x:c>
+      <x:c r="E16" t="str">
+        <x:v>All</x:v>
+      </x:c>
+      <x:c r="F16" t="str">
+        <x:v>Manual in setup, later generated from parser contract</x:v>
+      </x:c>
+      <x:c r="G16" t="str">
+        <x:v>Tower setup mapping</x:v>
+      </x:c>
+      <x:c r="H16" t="str">
+        <x:v>Must name source rows and dashboard surface</x:v>
+      </x:c>
+      <x:c r="I16" t="str">
+        <x:v>Explains why dashboard changed after an upload.</x:v>
+      </x:c>
+    </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
@@ -2131,6 +2729,18 @@
         <x:v>collection_owner</x:v>
       </x:c>
       <x:c r="K1" t="str">
+        <x:v>current_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>future_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
+        <x:v>dashboard_metric_family</x:v>
+      </x:c>
+      <x:c r="N1" t="str">
+        <x:v>dashboard_update_rule</x:v>
+      </x:c>
+      <x:c r="O1" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
@@ -2166,6 +2776,18 @@
         <x:v>Store Ops</x:v>
       </x:c>
       <x:c r="K2" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
+        <x:v>adoption</x:v>
+      </x:c>
+      <x:c r="N2" t="str">
+        <x:v>Refresh adoption tile and adoption pressure if active users remain below target.</x:v>
+      </x:c>
+      <x:c r="O2" t="str">
         <x:v>Copilot adoption evidence</x:v>
       </x:c>
     </x:row>
@@ -2199,6 +2821,18 @@
         <x:v>Enablement</x:v>
       </x:c>
       <x:c r="K3" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
+        <x:v>adoption</x:v>
+      </x:c>
+      <x:c r="N3" t="str">
+        <x:v>Refresh adoption blocker narrative after training completion is joined to eligible population.</x:v>
+      </x:c>
+      <x:c r="O3" t="str">
         <x:v>Manual roster join allowed</x:v>
       </x:c>
     </x:row>
@@ -2234,6 +2868,18 @@
         <x:v>Care Ops</x:v>
       </x:c>
       <x:c r="K4" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
+        <x:v>value_risk</x:v>
+      </x:c>
+      <x:c r="N4" t="str">
+        <x:v>Refresh value-lag scorecard and risk lens when containment trails target.</x:v>
+      </x:c>
+      <x:c r="O4" t="str">
         <x:v>Production AI workflow evidence</x:v>
       </x:c>
     </x:row>
@@ -2269,6 +2915,18 @@
         <x:v>Enterprise Services</x:v>
       </x:c>
       <x:c r="K5" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
+        <x:v>adoption</x:v>
+      </x:c>
+      <x:c r="N5" t="str">
+        <x:v>Refresh ServiceNow adoption pressure when deflection is below target or reopen rate rises.</x:v>
+      </x:c>
+      <x:c r="O5" t="str">
         <x:v>ServiceNow agent evidence</x:v>
       </x:c>
     </x:row>
@@ -2302,6 +2960,18 @@
         <x:v>FinOps</x:v>
       </x:c>
       <x:c r="K6" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
+        <x:v>foundation</x:v>
+      </x:c>
+      <x:c r="N6" t="str">
+        <x:v>Refresh evidence map and foundation gate when cost attribution coverage changes.</x:v>
+      </x:c>
+      <x:c r="O6" t="str">
         <x:v>Foundation evidence</x:v>
       </x:c>
     </x:row>
@@ -2337,6 +3007,18 @@
         <x:v>Product Ops</x:v>
       </x:c>
       <x:c r="K7" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="L7" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="M7" t="str">
+        <x:v>value</x:v>
+      </x:c>
+      <x:c r="N7" t="str">
+        <x:v>Refresh value tile after delivery cycle-time and release quality rows are committed.</x:v>
+      </x:c>
+      <x:c r="O7" t="str">
         <x:v>AI-led product development evidence</x:v>
       </x:c>
     </x:row>
@@ -2378,6 +3060,15 @@
         <x:v>source_system</x:v>
       </x:c>
       <x:c r="J1" t="str">
+        <x:v>current_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="K1" t="str">
+        <x:v>future_refresh_cycle</x:v>
+      </x:c>
+      <x:c r="L1" t="str">
+        <x:v>dashboard_update_rule</x:v>
+      </x:c>
+      <x:c r="M1" t="str">
         <x:v>notes</x:v>
       </x:c>
     </x:row>
@@ -2410,6 +3101,15 @@
         <x:v>Contract register</x:v>
       </x:c>
       <x:c r="J2" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="K2" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="L2" t="str">
+        <x:v>Refresh 90-day renewal, contract lens, and Source handoff after renewal date/value is validated.</x:v>
+      </x:c>
+      <x:c r="M2" t="str">
         <x:v>Renewal inside 90 days</x:v>
       </x:c>
     </x:row>
@@ -2442,6 +3142,15 @@
         <x:v>GitHub + procurement</x:v>
       </x:c>
       <x:c r="J3" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="K3" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="L3" t="str">
+        <x:v>Refresh dependency and adoption context after usage and renewal rows are joined.</x:v>
+      </x:c>
+      <x:c r="M3" t="str">
         <x:v>Scaled developer rollout</x:v>
       </x:c>
     </x:row>
@@ -2474,6 +3183,15 @@
         <x:v>SAP contract register</x:v>
       </x:c>
       <x:c r="J4" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="K4" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="L4" t="str">
+        <x:v>Refresh ERP-agent dependency and renewal pressure after contract and process evidence are validated.</x:v>
+      </x:c>
+      <x:c r="M4" t="str">
         <x:v>ERP workflow agent</x:v>
       </x:c>
     </x:row>
@@ -2506,6 +3224,15 @@
         <x:v>ServiceNow contract register</x:v>
       </x:c>
       <x:c r="J5" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="K5" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="L5" t="str">
+        <x:v>Refresh ServiceNow dependency card after contract and ITSM usage evidence are joined.</x:v>
+      </x:c>
+      <x:c r="M5" t="str">
         <x:v>Enterprise service agent</x:v>
       </x:c>
     </x:row>
@@ -2538,6 +3265,15 @@
         <x:v>Vendor contract register</x:v>
       </x:c>
       <x:c r="J6" t="str">
+        <x:v>Weekly</x:v>
+      </x:c>
+      <x:c r="K6" t="str">
+        <x:v>Daily API/export</x:v>
+      </x:c>
+      <x:c r="L6" t="str">
+        <x:v>Refresh AI-led product development dependency after usage, delivery, and spend evidence are joined.</x:v>
+      </x:c>
+      <x:c r="M6" t="str">
         <x:v>AI-led product development</x:v>
       </x:c>
     </x:row>

</xml_diff>

<commit_message>
Set Tower workbook cell alignment
</commit_message>
<xml_diff>
--- a/docs/build/tower-ai-program-template/AI_Program_Tracking_Template_Tower_v1.xlsx
+++ b/docs/build/tower-ai-program-template/AI_Program_Tracking_Template_Tower_v1.xlsx
@@ -2,35 +2,35 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="Reb1c5b05bc674e99"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CIO Readout" sheetId="2" r:id="R67ce749f77584709"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Instructions" sheetId="3" r:id="R5f6374a3e6ae4cbe"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import PMO Register" sheetId="4" r:id="Rec35a2b3dae1401e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Finance KPIs" sheetId="5" r:id="Rdd935834deb44334"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import M365 Copilot" sheetId="6" r:id="R70fe7b96f4c8423a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Dev AI Tools" sheetId="7" r:id="R037fa00873ca4e7b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import CX Agent" sheetId="8" r:id="R0c1e61d9ed57482d"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import SAP ERP" sheetId="9" r:id="Rb998dedb6f054ac1"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Forecast ML" sheetId="10" r:id="R718dda4fa63f4423"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import FinOps Gateway" sheetId="11" r:id="Rba2f0aacfbe54245"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Personalization" sheetId="12" r:id="R202abd54ae584ab0"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Procurement" sheetId="13" r:id="Refd0013a72ad42c6"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Governance" sheetId="14" r:id="R306f3d7fb76a44c7"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Stakeholder" sheetId="15" r:id="R8cfb5a8d0e374956"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Scenarios" sheetId="16" r:id="R89a4fbf086cd4194"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Upload Manifest" sheetId="17" r:id="Rfd187cf2496340b3"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Register" sheetId="18" r:id="R63a3b32749f44e57"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category Playbooks" sheetId="19" r:id="R1f6f70ff8b1f4c5b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tower Setup Upload" sheetId="20" r:id="Rf9e4bbe9218542ab"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Dictionary" sheetId="21" r:id="Ra81dc77e27314b3a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI History" sheetId="22" r:id="R4763207512c0409b"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendors and Renewals" sheetId="23" r:id="Ra254bdc2bc5e4570"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="24" r:id="R528347758dba478c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stakeholder Notes" sheetId="25" r:id="R0db528e910674112"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="26" r:id="Rc7302bb353c74410"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard Feed Map" sheetId="27" r:id="R5d889bf042b14c65"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tower Mapping" sheetId="28" r:id="R0934e7fbdb0d4e8e"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="29" r:id="Ra9eeddd7e1de4485"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="1" r:id="R3f372a06d2e84cbd"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="CIO Readout" sheetId="2" r:id="R9dc050703232406b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Instructions" sheetId="3" r:id="R3a03ccbd52624d68"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import PMO Register" sheetId="4" r:id="R71babf4b99f14cd8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Finance KPIs" sheetId="5" r:id="R0e4f8413e40747ef"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import M365 Copilot" sheetId="6" r:id="R9331d4fdd2bd4933"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Dev AI Tools" sheetId="7" r:id="R42e1e00a678a41fb"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import CX Agent" sheetId="8" r:id="R662bd85b29ca4d0d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import SAP ERP" sheetId="9" r:id="R94c3232b6dd9473f"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Forecast ML" sheetId="10" r:id="R5b1bbff2cdff4471"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import FinOps Gateway" sheetId="11" r:id="Rd129bce8dea74a9b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Personalization" sheetId="12" r:id="R290f22ae2bc149cf"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Procurement" sheetId="13" r:id="R8257bb73e78645b3"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Governance" sheetId="14" r:id="R176fe3d83edc4369"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Stakeholder" sheetId="15" r:id="R3776f73814b749a9"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Import Scenarios" sheetId="16" r:id="R31a0b02a8411455d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Source Upload Manifest" sheetId="17" r:id="R683d799851fb4fb5"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Program Register" sheetId="18" r:id="Rb3b56b4fdde54c19"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Category Playbooks" sheetId="19" r:id="Ra4bc9bcf478d40c1"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tower Setup Upload" sheetId="20" r:id="Rd86a1d81586440a6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Field Dictionary" sheetId="21" r:id="R3a5391841e88454e"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="KPI History" sheetId="22" r:id="Rf925ea6cf6c14c50"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Vendors and Renewals" sheetId="23" r:id="R35fdfc5f43174e58"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Decisions" sheetId="24" r:id="R77a4853c14734be6"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Stakeholder Notes" sheetId="25" r:id="Rf99b09cb34c4479d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Scenarios" sheetId="26" r:id="R29419b70621b4173"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Dashboard Feed Map" sheetId="27" r:id="R1b4fc2c9b37d4858"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Tower Mapping" sheetId="28" r:id="Rd0bbbf611b034448"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Data Quality" sheetId="29" r:id="R6924e951c69144ee"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -212,40 +212,40 @@
       <x:alignment horizontal="left" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="8" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="7" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -274,22 +274,22 @@
       <x:alignment horizontal="left" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="9" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
     </x:xf>
     <x:xf numFmtId="0" fontId="2" fillId="2" borderId="11" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="left" vertical="center" wrapText="1"/>
@@ -341,7 +341,7 @@
       </x:extLst>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
       <x:extLst>
         <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>
@@ -349,7 +349,7 @@
       </x:extLst>
     </x:xf>
     <x:xf numFmtId="0" fontId="1" fillId="0" borderId="10" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <x:alignment horizontal="left" vertical="top" wrapText="1"/>
+      <x:alignment horizontal="left" vertical="bottom" wrapText="1"/>
       <x:extLst>
         <x:ext uri="{C7286773-470A-42A8-94C5-96B5CB345126}">
           <xfpb:xfComplement xmlns:xfpb="http://schemas.microsoft.com/office/spreadsheetml/2022/featurepropertybag" i="0"/>

</xml_diff>